<commit_message>
Ordering: type-to-search customer picker, ship-to from customer on file (editable), Add New Customer with accounting email; customer addresses + QuickBooks id
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KWUUUp9o1XpyrtwvsW5QT6
</commit_message>
<xml_diff>
--- a/public/templates/customers-template.xlsx
+++ b/public/templates/customers-template.xlsx
@@ -482,16 +482,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -512,22 +516,42 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Billing Address</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Shipping Address</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>State</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>QuickBooks ID</t>
         </is>
       </c>
     </row>
@@ -549,24 +573,40 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>405-555-0100</t>
+          <t>Pat Smith</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>office@example.com</t>
+          <t>405-555-0100</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>office@example.com</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>100 Main St, Oklahoma City, OK 73102</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>4700 S Council Rd, Oklahoma City, OK 73179</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -9586,6 +9626,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -9610,10 +9651,11 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Customers are matched by Account No (or by name if there is no account number), so re-importing updates them.</t>
+          <t>Customers are matched by QuickBooks ID, then Account No, then name, so re-importing updates them. Shipping Address fills in the ship-to on the order screen (Billing Address is used if it is blank).</t>
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sales reps, invoice prices and sales goals: each customer gets a sales rep (Admin > Customers, one at a time, ticked in bulk, or from the import's "Sales Rep" column) and every order credits that rep; the order desk enters each item's price from the invoice with the Sales Order # and Invoice # (required for spray foam, fiberglass and other customer-priced items), so order totals, the PDF and sales use real prices; monthly sales goals by product group (Foam, Fiberglass, PPE, Roof Coatings & Sealants, Gun & Parts, Intumescent Coatings, Sealants / Adhesives, Tools Accessories & Supplies) for sales reps (their customers) and warehouse managers (their location), set in Admin > Sales goals, tracked on Home and in /sales-goals; categories pick their goal group. Jump back in no longer shows deleted, cancelled or completed orders. Needs database update 0028.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KWUUUp9o1XpyrtwvsW5QT6
</commit_message>
<xml_diff>
--- a/public/templates/customers-template.xlsx
+++ b/public/templates/customers-template.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1000"/>
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -554,6 +555,11 @@
           <t>QuickBooks ID</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -607,6 +613,11 @@
         </is>
       </c>
       <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Rep name or email</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -9610,7 +9621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9626,7 +9637,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -9655,7 +9665,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
@@ -9824,6 +9833,23 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>The AMBIT sales rep's name or email (as in Admin → Accounts). Their orders count toward that rep's sales goals.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>